<commit_message>
Update bug report and test cases
</commit_message>
<xml_diff>
--- a/manual-testing/barbora-webshop-testing/bug-report/Bug report.xlsx
+++ b/manual-testing/barbora-webshop-testing/bug-report/Bug report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96c6bdc0c0427c4e/Desktop/Martins/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96c6bdc0c0427c4e/Desktop/qa-portfolio/manual-testing/barbora-webshop-testing/bug-report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="145" documentId="8_{C318B0C1-86A5-46CD-87BB-F2A308CCABB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B93F3723-B0A2-491D-9545-A494B3D1A025}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{C318B0C1-86A5-46CD-87BB-F2A308CCABB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A5DECAE-08D3-44FE-BE7E-52831393C74E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CA6AADD1-F631-492F-80A4-DD9A62D3DE41}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="79">
   <si>
     <t>Test type</t>
   </si>
@@ -215,45 +215,18 @@
     <t>Products and buttons are visible, but the totals are not shown</t>
   </si>
   <si>
-    <t>Enter an incorrect e-mail address missing the last letter of the top-level domain (Test Data: "loyalcustomer123321@gmail.co")</t>
-  </si>
-  <si>
-    <t>Enter e-mail address (Test Data: "loyalcustomer123312@gmail.com")</t>
-  </si>
-  <si>
     <t>Enter a name and surname containing long vowels and diacritical marks used in the Latvian language (Test Data: name and surname: "Jānis Bērziņš")</t>
   </si>
   <si>
-    <t>Enter correct name, surname, phone number and password (Test Data: name and surname: "Janis Berzins", phone: "25427xxx", password: "JanisBerzins1")</t>
-  </si>
-  <si>
     <t>Choose city from the drop-down (Test Data: "Riga")</t>
   </si>
   <si>
-    <t>Choose street from the drop-down (Test Data: "Latgales iela xxx, LV-xxxx")</t>
-  </si>
-  <si>
     <t>Enter apartment number using letters (Test Data: "asdasd")</t>
   </si>
   <si>
     <t>Enter flat number longer than 10 symbols (Test Data: "yutqweuwqeyuqweyuqweqtuweq")</t>
   </si>
   <si>
-    <t>Enter incorrect e-mail address containing two "@" special symbols (Test Data: "loyal@customer123312@gmail.com")</t>
-  </si>
-  <si>
-    <t>Enter correct password (TestData: "JanisBerzins1")</t>
-  </si>
-  <si>
-    <t>Enter correct password (Test Data: "JanisBerzins1")</t>
-  </si>
-  <si>
-    <t>Enter correct e-mail address (Test Data: "loyalcustomer123321@gmail.com")</t>
-  </si>
-  <si>
-    <t>Enter incorrect password (Test Data: "Janis1234")</t>
-  </si>
-  <si>
     <t xml:space="preserve">Test Object: </t>
   </si>
   <si>
@@ -270,13 +243,43 @@
   </si>
   <si>
     <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/142.0.0.0 Safari/537.36</t>
+  </si>
+  <si>
+    <t>Enter an incorrect e-mail address missing the last letter of the top-level domain (Test Data: "registered.test.user@example.co")</t>
+  </si>
+  <si>
+    <t>Enter e-mail address (Test Data: "registered.test.user@example.com")</t>
+  </si>
+  <si>
+    <t>Enter correct name, surname, phone number and password (Test Data: name and surname: "Janis Berzins", phone: correct phone number, password: "ValidTestPassword123!")</t>
+  </si>
+  <si>
+    <t>Choose street from the drop-down (Test Data: "Vidzemes iela xxx, LV-xxxx")</t>
+  </si>
+  <si>
+    <t>Enter incorrect e-mail address containing two "@" special symbols (Test Data: "registered.test.user@example.com")</t>
+  </si>
+  <si>
+    <t>Enter correct password (TestData: "ValidTestPassword123!")</t>
+  </si>
+  <si>
+    <t>Enter incorrect e-mail address containing two "@" special symbols (Test Data: "registered.test@user@example.com")</t>
+  </si>
+  <si>
+    <t>Enter correct password (Test Data: "ValidTestPassword123!")</t>
+  </si>
+  <si>
+    <t>Enter correct e-mail address (Test Data: "registered.test.user@example.com")</t>
+  </si>
+  <si>
+    <t>Enter incorrect password (Test Data: "InvalidPassword123!")</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,13 +353,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -692,7 +695,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C76855-A9BA-48C1-BD0F-9C6CCBB8AB37}">
   <dimension ref="A1:I87"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" customWidth="1"/>
@@ -705,57 +708,57 @@
     <col min="9" max="9" width="18.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="B7" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
@@ -768,56 +771,56 @@
       <c r="E8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>14</v>
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+        <v>69</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="12" spans="1:9">
-      <c r="B12" s="7" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>8</v>
       </c>
@@ -830,92 +833,92 @@
       <c r="E13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="2:9">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
+        <v>59</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="20" spans="2:9">
-      <c r="B20" s="7" t="s">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="2:9">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
         <v>8</v>
       </c>
@@ -928,140 +931,140 @@
       <c r="E21" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="2:9">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" s="5"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="F22" s="6"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="2:9">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="2:9">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="2:9">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F25" s="5"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
+        <v>71</v>
+      </c>
+      <c r="F25" s="6"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
       <c r="I25" s="4"/>
     </row>
-    <row r="26" spans="2:9">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="F26" s="6"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
       <c r="I26" s="4"/>
     </row>
-    <row r="27" spans="2:9">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F27" s="5"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="F27" s="6"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
       <c r="I27" s="4"/>
     </row>
-    <row r="28" spans="2:9">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" s="5"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
+        <v>61</v>
+      </c>
+      <c r="F28" s="6"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="4"/>
     </row>
-    <row r="29" spans="2:9">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
       <c r="I29" s="4"/>
     </row>
-    <row r="32" spans="2:9">
-      <c r="B32" s="7" t="s">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E32" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G32" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H32" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I32" s="7" t="s">
+      <c r="I32" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="2:9">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B33" s="4" t="s">
         <v>8</v>
       </c>
@@ -1074,150 +1077,150 @@
       <c r="E33" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="G33" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I33" s="4"/>
     </row>
-    <row r="34" spans="2:9">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
       <c r="E34" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="7"/>
       <c r="I34" s="4"/>
     </row>
-    <row r="35" spans="2:9">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="7"/>
       <c r="I35" s="4"/>
     </row>
-    <row r="36" spans="2:9">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
       <c r="E36" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="7"/>
       <c r="I36" s="4"/>
     </row>
-    <row r="37" spans="2:9">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
       <c r="E37" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="6"/>
+        <v>71</v>
+      </c>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="7"/>
       <c r="I37" s="4"/>
     </row>
-    <row r="38" spans="2:9">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="7"/>
       <c r="I38" s="4"/>
     </row>
-    <row r="39" spans="2:9">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
       <c r="E39" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="7"/>
       <c r="I39" s="4"/>
     </row>
-    <row r="40" spans="2:9">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
       <c r="E40" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="6"/>
+        <v>62</v>
+      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="7"/>
       <c r="I40" s="4"/>
     </row>
-    <row r="41" spans="2:9">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="7"/>
       <c r="I41" s="4"/>
     </row>
-    <row r="42" spans="2:9">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="2:9">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="2:9">
-      <c r="B44" s="7" t="s">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B44" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F44" s="7" t="s">
+      <c r="F44" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G44" s="7" t="s">
+      <c r="G44" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H44" s="7" t="s">
+      <c r="H44" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I44" s="7" t="s">
+      <c r="I44" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="2:9">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B45" s="4" t="s">
         <v>29</v>
       </c>
@@ -1230,56 +1233,56 @@
       <c r="E45" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="F45" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G45" s="6" t="s">
+      <c r="G45" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="H45" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I45" s="4"/>
     </row>
-    <row r="46" spans="2:9">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
       <c r="E46" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
       <c r="I46" s="4"/>
     </row>
-    <row r="50" spans="2:9">
-      <c r="B50" s="7" t="s">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B50" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D50" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F50" s="7" t="s">
+      <c r="F50" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G50" s="7" t="s">
+      <c r="G50" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H50" s="7" t="s">
+      <c r="H50" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I50" s="7" t="s">
+      <c r="I50" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="2:9">
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B51" s="4" t="s">
         <v>29</v>
       </c>
@@ -1292,80 +1295,80 @@
       <c r="E51" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="F51" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G51" s="5" t="s">
+      <c r="G51" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H51" s="6" t="s">
+      <c r="H51" s="7" t="s">
         <v>14</v>
       </c>
       <c r="I51" s="4"/>
     </row>
-    <row r="52" spans="2:9">
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
       <c r="E52" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="6"/>
+        <v>73</v>
+      </c>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="7"/>
       <c r="I52" s="4"/>
     </row>
-    <row r="53" spans="2:9">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="6"/>
+        <v>74</v>
+      </c>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="7"/>
       <c r="I53" s="4"/>
     </row>
-    <row r="54" spans="2:9">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="7"/>
       <c r="I54" s="4"/>
     </row>
-    <row r="57" spans="2:9">
-      <c r="B57" s="7" t="s">
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B57" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C57" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D57" s="7" t="s">
+      <c r="D57" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E57" s="7" t="s">
+      <c r="E57" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F57" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G57" s="7" t="s">
+      <c r="G57" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H57" s="7" t="s">
+      <c r="H57" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I57" s="7" t="s">
+      <c r="I57" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="2:9">
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B58" s="4" t="s">
         <v>29</v>
       </c>
@@ -1378,80 +1381,80 @@
       <c r="E58" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="F58" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G58" s="5" t="s">
+      <c r="G58" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H58" s="6" t="s">
+      <c r="H58" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I58" s="4"/>
     </row>
-    <row r="59" spans="2:9">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
       <c r="E59" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="6"/>
+        <v>75</v>
+      </c>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
+      <c r="H59" s="7"/>
       <c r="I59" s="4"/>
     </row>
-    <row r="60" spans="2:9">
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
       <c r="E60" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
-      <c r="H60" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="7"/>
       <c r="I60" s="4"/>
     </row>
-    <row r="61" spans="2:9">
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="7"/>
       <c r="I61" s="4"/>
     </row>
-    <row r="65" spans="2:9">
-      <c r="B65" s="7" t="s">
+    <row r="65" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B65" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="C65" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D65" s="7" t="s">
+      <c r="D65" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E65" s="7" t="s">
+      <c r="E65" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F65" s="7" t="s">
+      <c r="F65" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G65" s="7" t="s">
+      <c r="G65" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H65" s="7" t="s">
+      <c r="H65" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I65" s="7" t="s">
+      <c r="I65" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="2:9">
+    <row r="66" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B66" s="4" t="s">
         <v>29</v>
       </c>
@@ -1464,109 +1467,109 @@
       <c r="E66" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F66" s="6" t="s">
+      <c r="F66" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G66" s="6" t="s">
+      <c r="G66" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H66" s="6" t="s">
+      <c r="H66" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I66" s="4"/>
     </row>
-    <row r="67" spans="2:9">
+    <row r="67" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
+        <v>77</v>
+      </c>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
       <c r="I67" s="4"/>
     </row>
-    <row r="68" spans="2:9">
+    <row r="68" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F68" s="6"/>
-      <c r="G68" s="6"/>
-      <c r="H68" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7"/>
       <c r="I68" s="4"/>
     </row>
-    <row r="69" spans="2:9">
+    <row r="69" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
       <c r="E69" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F69" s="6"/>
-      <c r="G69" s="6"/>
-      <c r="H69" s="6"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7"/>
       <c r="I69" s="4"/>
     </row>
-    <row r="70" spans="2:9">
+    <row r="70" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
       <c r="E70" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F70" s="6"/>
-      <c r="G70" s="6"/>
-      <c r="H70" s="6"/>
+      <c r="F70" s="7"/>
+      <c r="G70" s="7"/>
+      <c r="H70" s="7"/>
       <c r="I70" s="4"/>
     </row>
-    <row r="71" spans="2:9">
+    <row r="71" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F71" s="6"/>
-      <c r="G71" s="6"/>
-      <c r="H71" s="6"/>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="7"/>
       <c r="I71" s="4"/>
     </row>
-    <row r="72" spans="2:9">
+    <row r="72" spans="2:9" x14ac:dyDescent="0.3">
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
     </row>
-    <row r="74" spans="2:9">
-      <c r="B74" s="7" t="s">
+    <row r="74" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B74" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="C74" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D74" s="7" t="s">
+      <c r="D74" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E74" s="7" t="s">
+      <c r="E74" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F74" s="7" t="s">
+      <c r="F74" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G74" s="7" t="s">
+      <c r="G74" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H74" s="7" t="s">
+      <c r="H74" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I74" s="7" t="s">
+      <c r="I74" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="2:9">
+    <row r="75" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B75" s="4" t="s">
         <v>29</v>
       </c>
@@ -1579,80 +1582,80 @@
       <c r="E75" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F75" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G75" s="5" t="s">
+      <c r="G75" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H75" s="6" t="s">
+      <c r="H75" s="7" t="s">
         <v>14</v>
       </c>
       <c r="I75" s="4"/>
     </row>
-    <row r="76" spans="2:9">
+    <row r="76" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
       <c r="E76" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="6"/>
+        <v>77</v>
+      </c>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6"/>
+      <c r="H76" s="7"/>
       <c r="I76" s="4"/>
     </row>
-    <row r="77" spans="2:9">
+    <row r="77" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5"/>
-      <c r="H77" s="6"/>
+        <v>78</v>
+      </c>
+      <c r="F77" s="6"/>
+      <c r="G77" s="6"/>
+      <c r="H77" s="7"/>
       <c r="I77" s="4"/>
     </row>
-    <row r="78" spans="2:9">
+    <row r="78" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5"/>
-      <c r="H78" s="6"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="6"/>
+      <c r="H78" s="7"/>
       <c r="I78" s="4"/>
     </row>
-    <row r="83" spans="2:9">
-      <c r="B83" s="7" t="s">
+    <row r="83" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B83" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C83" s="7" t="s">
+      <c r="C83" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D83" s="7" t="s">
+      <c r="D83" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E83" s="7" t="s">
+      <c r="E83" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F83" s="7" t="s">
+      <c r="F83" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G83" s="7" t="s">
+      <c r="G83" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H83" s="7" t="s">
+      <c r="H83" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I83" s="7" t="s">
+      <c r="I83" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="2:9">
+    <row r="84" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B84" s="4" t="s">
         <v>51</v>
       </c>
@@ -1665,85 +1668,85 @@
       <c r="E84" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F84" s="6" t="s">
+      <c r="F84" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G84" s="6" t="s">
+      <c r="G84" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="H84" s="6" t="s">
+      <c r="H84" s="7" t="s">
         <v>14</v>
       </c>
       <c r="I84" s="4"/>
     </row>
-    <row r="85" spans="2:9">
+    <row r="85" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
       <c r="D85" s="4"/>
       <c r="E85" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="F85" s="6"/>
-      <c r="G85" s="6"/>
-      <c r="H85" s="6"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="7"/>
+      <c r="H85" s="7"/>
       <c r="I85" s="4"/>
     </row>
-    <row r="86" spans="2:9">
+    <row r="86" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
       <c r="D86" s="4"/>
       <c r="E86" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F86" s="6"/>
-      <c r="G86" s="6"/>
-      <c r="H86" s="6"/>
+      <c r="F86" s="7"/>
+      <c r="G86" s="7"/>
+      <c r="H86" s="7"/>
       <c r="I86" s="4"/>
     </row>
-    <row r="87" spans="2:9">
+    <row r="87" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
       <c r="D87" s="4"/>
       <c r="E87" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F87" s="6"/>
-      <c r="G87" s="6"/>
-      <c r="H87" s="6"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="7"/>
+      <c r="H87" s="7"/>
       <c r="I87" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="F13:F17"/>
+    <mergeCell ref="G13:G17"/>
+    <mergeCell ref="H13:H17"/>
+    <mergeCell ref="F21:F29"/>
+    <mergeCell ref="G21:G29"/>
+    <mergeCell ref="H21:H29"/>
+    <mergeCell ref="F33:F41"/>
+    <mergeCell ref="G33:G41"/>
+    <mergeCell ref="H33:H41"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="F51:F54"/>
+    <mergeCell ref="G51:G54"/>
+    <mergeCell ref="H51:H54"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="F66:F71"/>
+    <mergeCell ref="G66:G71"/>
+    <mergeCell ref="H66:H71"/>
     <mergeCell ref="F75:F78"/>
     <mergeCell ref="G75:G78"/>
     <mergeCell ref="H75:H78"/>
     <mergeCell ref="F84:F87"/>
     <mergeCell ref="G84:G87"/>
     <mergeCell ref="H84:H87"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="G58:G61"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="F66:F71"/>
-    <mergeCell ref="G66:G71"/>
-    <mergeCell ref="H66:H71"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="H45:H46"/>
-    <mergeCell ref="F51:F54"/>
-    <mergeCell ref="G51:G54"/>
-    <mergeCell ref="H51:H54"/>
-    <mergeCell ref="F21:F29"/>
-    <mergeCell ref="G21:G29"/>
-    <mergeCell ref="H21:H29"/>
-    <mergeCell ref="F33:F41"/>
-    <mergeCell ref="G33:G41"/>
-    <mergeCell ref="H33:H41"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="F13:F17"/>
-    <mergeCell ref="G13:G17"/>
-    <mergeCell ref="H13:H17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>